<commit_message>
Update BOM.xlsx, PartsLocation.pptx indicates F1 as jumper.
</commit_message>
<xml_diff>
--- a/hardware/BOM.xlsx
+++ b/hardware/BOM.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\192.168.0.114\momose\FlukeNIC\hardware\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\192.168.0.115\momose\FlukeNIC\hardware\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85801760-D399-46A3-9182-E214F00E0CEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E840A80B-B484-40B5-8E87-09C94EF3B6C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1005" yWindow="825" windowWidth="21600" windowHeight="11535" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="761" yWindow="761" windowWidth="24955" windowHeight="20540" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FlukeNIC_BOM" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="97">
   <si>
     <t>Qty</t>
   </si>
@@ -159,14 +159,6 @@
     <phoneticPr fontId="2"/>
   </si>
   <si>
-    <t>MF-RX040/72-0</t>
-    <phoneticPr fontId="2"/>
-  </si>
-  <si>
-    <t>Resettable fuse 0.4A</t>
-    <phoneticPr fontId="2"/>
-  </si>
-  <si>
     <t>Generic resistor</t>
     <phoneticPr fontId="2"/>
   </si>
@@ -352,6 +344,10 @@
   </si>
   <si>
     <t>Voltage reg 3.3V, Low drop, Package TO-252-3</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>Not use, use jumper instead</t>
     <phoneticPr fontId="2"/>
   </si>
 </sst>
@@ -717,7 +713,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I43"/>
-  <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
+  <sheetFormatPr defaultRowHeight="12.9" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="3.125" customWidth="1"/>
     <col min="2" max="2" width="31.625" customWidth="1"/>
@@ -731,7 +727,7 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A1" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.15">
@@ -761,7 +757,7 @@
         <v>32</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="F3" s="1"/>
       <c r="I3" s="1"/>
@@ -856,7 +852,7 @@
         <v>2</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>39</v>
@@ -904,11 +900,9 @@
         <v>1</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="E12" s="1" t="s">
-        <v>43</v>
-      </c>
+        <v>96</v>
+      </c>
+      <c r="E12" s="1"/>
       <c r="F12" s="1"/>
       <c r="H12" s="1"/>
       <c r="I12" s="1"/>
@@ -924,7 +918,7 @@
         <v>14</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="F13" s="1"/>
       <c r="I13" s="1"/>
@@ -940,7 +934,7 @@
         <v>16</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="F14" s="1"/>
       <c r="I14" s="1"/>
@@ -956,7 +950,7 @@
         <v>5</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="F15" s="1"/>
       <c r="I15" s="1"/>
@@ -969,10 +963,10 @@
         <v>1</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="F16" s="1"/>
       <c r="H16" s="1"/>
@@ -986,10 +980,10 @@
         <v>1</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="F17" s="1"/>
       <c r="H17" s="1"/>
@@ -1036,7 +1030,7 @@
         <v>27</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="F20" s="1"/>
       <c r="H20" s="1"/>
@@ -1044,7 +1038,7 @@
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.15">
       <c r="A22" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.15">
@@ -1063,7 +1057,7 @@
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.15">
       <c r="B24" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C24" s="1">
         <v>7</v>
@@ -1072,12 +1066,12 @@
         <v>0.1</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.15">
       <c r="B25" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="C25" s="1">
         <v>2</v>
@@ -1086,7 +1080,7 @@
         <v>0.01</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.15">
@@ -1097,127 +1091,127 @@
         <v>1</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.15">
       <c r="B27" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C27" s="1">
+        <v>1</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E27" s="1" t="s">
         <v>52</v>
-      </c>
-      <c r="C27" s="1">
-        <v>1</v>
-      </c>
-      <c r="D27" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="E27" s="1" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.15">
       <c r="B28" s="1" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C28" s="1">
         <v>1</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.15">
       <c r="B29" s="1" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C29" s="1">
         <v>1</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.15">
       <c r="B30" s="1" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C30" s="1">
         <v>1</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.15">
       <c r="B31" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C31" s="1">
         <v>4</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.15">
       <c r="B32" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C32" s="1">
+        <v>1</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="E32" s="1" t="s">
         <v>64</v>
-      </c>
-      <c r="C32" s="1">
-        <v>1</v>
-      </c>
-      <c r="D32" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="E32" s="1" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="33" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B33" s="1" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C33" s="1">
         <v>2</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="34" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B34" s="1" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="C34" s="1">
         <v>9</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="35" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B35" s="1" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C35" s="1">
         <v>3</v>
@@ -1226,26 +1220,26 @@
         <v>470</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="36" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B36" s="1" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C36" s="1">
         <v>2</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="37" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B37" s="1" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C37" s="1">
         <v>2</v>
@@ -1254,21 +1248,21 @@
         <v>14</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="38" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B38" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C38" s="1">
         <v>2</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="39" spans="2:5" x14ac:dyDescent="0.15">
@@ -1279,10 +1273,10 @@
         <v>1</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="40" spans="2:5" x14ac:dyDescent="0.15">
@@ -1293,10 +1287,10 @@
         <v>1</v>
       </c>
       <c r="D40" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="E40" s="1" t="s">
         <v>92</v>
-      </c>
-      <c r="E40" s="1" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="41" spans="2:5" x14ac:dyDescent="0.15">
@@ -1307,10 +1301,10 @@
         <v>1</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="42" spans="2:5" x14ac:dyDescent="0.15">
@@ -1321,24 +1315,24 @@
         <v>1</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="43" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B43" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C43" s="1">
+        <v>1</v>
+      </c>
+      <c r="D43" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="E43" s="1" t="s">
         <v>84</v>
-      </c>
-      <c r="C43" s="1">
-        <v>1</v>
-      </c>
-      <c r="D43" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="E43" s="1" t="s">
-        <v>86</v>
       </c>
     </row>
   </sheetData>

</xml_diff>